<commit_message>
Continuing exploring Ron's data
</commit_message>
<xml_diff>
--- a/data/from-Ron/Ron-data_columns.xlsx
+++ b/data/from-Ron/Ron-data_columns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eltnmsu-my.sharepoint.com/personal/lossanna_nmsu_edu/Documents/Documents/04_LDC-LTDL/LDC-LTDL/data/from-Ron/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="411" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FC57CF2-0BEA-409D-9568-D6B4BBAC8835}"/>
+  <xr:revisionPtr revIDLastSave="485" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59F39C67-4CDF-4963-BEC3-430F6649A60E}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="1620" windowWidth="20376" windowHeight="12096" activeTab="1" xr2:uid="{180FE257-6980-4323-B5A2-AB4BD0017CAE}"/>
+    <workbookView xWindow="22908" yWindow="1596" windowWidth="20424" windowHeight="12144" activeTab="1" xr2:uid="{180FE257-6980-4323-B5A2-AB4BD0017CAE}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="120">
   <si>
     <t>Column</t>
   </si>
@@ -259,6 +259,144 @@
   </si>
   <si>
     <t>Major Land Resource Area (symbol)</t>
+  </si>
+  <si>
+    <t>Prj_ID</t>
+  </si>
+  <si>
+    <t>Trt_ID</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>init_month</t>
+  </si>
+  <si>
+    <t>init_day</t>
+  </si>
+  <si>
+    <t>init_yr</t>
+  </si>
+  <si>
+    <t>comp_month</t>
+  </si>
+  <si>
+    <t>comp_day</t>
+  </si>
+  <si>
+    <t>comp_yr</t>
+  </si>
+  <si>
+    <t>LTDL Treatment_Info.csv</t>
+  </si>
+  <si>
+    <t>LTDL Project_Info.csv</t>
+  </si>
+  <si>
+    <t>NA; 1-8</t>
+  </si>
+  <si>
+    <t>LTDL Project ID</t>
+  </si>
+  <si>
+    <t>LTDL Treatment ID</t>
+  </si>
+  <si>
+    <t>If treatment was successful</t>
+  </si>
+  <si>
+    <t>Month that treatment was initiated</t>
+  </si>
+  <si>
+    <t>Day that treatment was initiated</t>
+  </si>
+  <si>
+    <t>Year that treatment was initiated</t>
+  </si>
+  <si>
+    <t>Month that treatment was completed</t>
+  </si>
+  <si>
+    <t>Day that treatment was completed</t>
+  </si>
+  <si>
+    <t>Year that treament was completed</t>
+  </si>
+  <si>
+    <t>Trt_Type_M</t>
+  </si>
+  <si>
+    <t>Treatment type (major)</t>
+  </si>
+  <si>
+    <t>Trt_Type_S</t>
+  </si>
+  <si>
+    <t>Treatment type (sub)</t>
+  </si>
+  <si>
+    <t>treatment</t>
+  </si>
+  <si>
+    <t>Treatment category that Ron developed</t>
+  </si>
+  <si>
+    <t>11 options (includes NA)</t>
+  </si>
+  <si>
+    <t>20 options (includes NA)</t>
+  </si>
+  <si>
+    <t>71 options (includes NA)</t>
+  </si>
+  <si>
+    <t>rcnt_ptrt_yr</t>
+  </si>
+  <si>
+    <t>The year of the most recent something</t>
+  </si>
+  <si>
+    <t>trt_ptrt_dif</t>
+  </si>
+  <si>
+    <t>rcnt_ptrt_type</t>
+  </si>
+  <si>
+    <t>24 options</t>
+  </si>
+  <si>
+    <t>fire_occ</t>
+  </si>
+  <si>
+    <t>No fire; fire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If fire occurred </t>
+  </si>
+  <si>
+    <t>fire_binary</t>
+  </si>
+  <si>
+    <t>0; 1</t>
+  </si>
+  <si>
+    <t>Fire occurrence as binary</t>
+  </si>
+  <si>
+    <t>trt_control</t>
+  </si>
+  <si>
+    <t>no treatment; treated</t>
+  </si>
+  <si>
+    <t>If the plot was treated</t>
+  </si>
+  <si>
+    <t>trt_binary</t>
+  </si>
+  <si>
+    <t>Plot treatment as binary</t>
   </si>
 </sst>
 </file>
@@ -302,7 +440,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -312,13 +450,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -334,6 +465,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -706,7 +841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDAAED03-0683-4ECB-B284-67F38602FBED}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.44140625" bestFit="1" customWidth="1"/>
@@ -714,7 +849,7 @@
     <col min="3" max="3" width="21.21875" style="4" customWidth="1"/>
     <col min="4" max="4" width="44.88671875" style="4" customWidth="1"/>
     <col min="5" max="5" width="32.5546875" style="4" customWidth="1"/>
-    <col min="6" max="6" width="19" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -733,79 +868,74 @@
       <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="5" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="F2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="8"/>
-    </row>
-    <row r="4" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -816,10 +946,10 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -828,15 +958,15 @@
       <c r="E7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -845,197 +975,239 @@
       <c r="E8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" t="s">
         <v>5</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" t="s">
         <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" t="s">
         <v>41</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="A15" t="s">
         <v>42</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F15" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" t="s">
         <v>43</v>
+      </c>
+      <c r="B16" t="s">
+        <v>5</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="A17" t="s">
         <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="A18" t="s">
         <v>45</v>
+      </c>
+      <c r="B18" t="s">
+        <v>5</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="A19" t="s">
         <v>46</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="A20" t="s">
         <v>48</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" t="s">
         <v>54</v>
+      </c>
+      <c r="B21" t="s">
+        <v>5</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+      <c r="A22" t="s">
         <v>55</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" t="s">
         <v>56</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="F23" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" t="s">
         <v>57</v>
+      </c>
+      <c r="B24" t="s">
+        <v>5</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
+      <c r="A25" t="s">
         <v>59</v>
       </c>
+      <c r="B25" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="A26" t="s">
         <v>60</v>
+      </c>
+      <c r="B26" t="s">
+        <v>5</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>61</v>
@@ -1045,19 +1217,282 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="A27" t="s">
         <v>62</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+      <c r="A28" t="s">
         <v>64</v>
+      </c>
+      <c r="B28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>85</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F29" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>75</v>
+      </c>
+      <c r="B30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F30" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F31" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F32" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F33" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F34" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F35" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F36" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B37" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F37" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F38" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F39" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>107</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>109</v>
+      </c>
+      <c r="B44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>112</v>
+      </c>
+      <c r="B45" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>115</v>
+      </c>
+      <c r="B46" t="s">
+        <v>11</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>118</v>
+      </c>
+      <c r="B47" t="s">
+        <v>5</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>